<commit_message>
Remove DE macro features – US-only macro for methodological consistency
Design decision: DE Auftragseingangsindex (DE-010) and DE Produktionsindex (DE-011)
excluded from model. Revenue data consists exclusively of US customer transactions,
so DE domestic order intake has no direct causal pathway to US demand.
Including DE features risked spurious correlation (global cycle co-movement)
and overfitting on 33 observations.

Changes:
- notebooks/03: NON_STATIONARY and STATIONARY lists updated, design decision documented
- feature_matrix.csv: 38 cols -> 26 cols (12 DE lag features removed, 23 features total)
- Model retrained (04): 23 features, mean sMAPE 17.2% vs 19.3% before (-2.1pp)
- SHAP (05): US macro now clearly dominant macro group, no DE spurious signals
- Forecast (06): regenerated with new model
- SAC exports: updated feature group label DE->US_Macro, Appendix notes DE exclusion
</commit_message>
<xml_diff>
--- a/data/processed/DGE_Revenue_Forecast_XGBoost_2026.xlsx
+++ b/data/processed/DGE_Revenue_Forecast_XGBoost_2026.xlsx
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>2149267.75</v>
+        <v>2085386.75</v>
       </c>
     </row>
     <row r="4">
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="E4" s="8" t="n">
-        <v>2358887.25</v>
+        <v>2570691</v>
       </c>
     </row>
     <row r="5">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>2412206.75</v>
+        <v>2649504.25</v>
       </c>
     </row>
     <row r="6">
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="E6" s="8" t="n">
-        <v>2034275.75</v>
+        <v>2446111</v>
       </c>
     </row>
     <row r="7">
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>2266433</v>
+        <v>2271000.75</v>
       </c>
     </row>
     <row r="8">
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="E8" s="8" t="n">
-        <v>2021999.38</v>
+        <v>2491056.5</v>
       </c>
     </row>
     <row r="9">
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>1874729.38</v>
+        <v>2092556.25</v>
       </c>
     </row>
     <row r="10">
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="E10" s="8" t="n">
-        <v>1990016.88</v>
+        <v>2183507.75</v>
       </c>
     </row>
     <row r="11">
@@ -758,7 +758,7 @@
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>1817860.12</v>
+        <v>2337603.5</v>
       </c>
     </row>
     <row r="12">
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="E12" s="8" t="n">
-        <v>1823820.88</v>
+        <v>2118988.75</v>
       </c>
     </row>
     <row r="13">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>1823820.88</v>
+        <v>2071760.88</v>
       </c>
     </row>
     <row r="14">
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="E14" s="8" t="n">
-        <v>1442057.88</v>
+        <v>1791618.38</v>
       </c>
     </row>
     <row r="15">
@@ -837,13 +837,13 @@
         </is>
       </c>
       <c r="E15" s="10" t="n">
-        <v>24015375.88</v>
+        <v>27109785.75</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>2025 Actuals (reference)  |  YoY: -20.3%</t>
+          <t>2025 Actuals (reference)  |  YoY: -10.1%</t>
         </is>
       </c>
       <c r="E16" s="12" t="n">
@@ -866,11 +866,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -957,55 +957,79 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>XGBoost Regressor – trained on Apr 2023 to Dec 2025 (33 months)</t>
+          <t>XGBoost Regressor – trained on Apr 2023 to Dec 2025 (33 months, 23 features)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Method</t>
+          <t>Features</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Rolling one-step-ahead forecast; each prediction feeds next month's revenue lags</t>
+          <t>US macro lags (DGORDER, INDPRO), calendar, revenue AR/rolling</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Macro inputs</t>
+          <t>DE macro</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Carry-forward of Dec 2025 values from Jan 2026 onward (US data ends Dec 2025)</t>
+          <t>Excluded – no causal pathway from DE domestic orders to US customer revenue</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>B1/B2</t>
+          <t>Method</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>NOT subtracted – this is gross B3. Net B3 = Gross B3 - (B1 + B2) in SAC</t>
+          <t>Rolling one-step-ahead; each prediction feeds next month's revenue lags</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
+          <t>Macro inputs</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Carry-forward of Dec 2025 values from Jan 2026 onward</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>B1/B2</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>NOT subtracted – gross B3. Net B3 = Gross B3 - (B1+B2) in SAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
           <t>Limitation</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Synthetic data basis – absolute values demonstrate methodology, not calibrated forecast</t>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Synthetic data basis – absolute values demonstrate methodology</t>
         </is>
       </c>
     </row>

</xml_diff>